<commit_message>
chore: second run on 500
</commit_message>
<xml_diff>
--- a/data/output/authors_junk_names_elastic.xlsx
+++ b/data/output/authors_junk_names_elastic.xlsx
@@ -55,15 +55,15 @@
     <t>belongs_to</t>
   </si>
   <si>
+    <t>2025-11-15T14:20:59Z</t>
+  </si>
+  <si>
+    <t>2025-11-14T19:56:55Z</t>
+  </si>
+  <si>
     <t>2025-11-15T03:02:46Z</t>
   </si>
   <si>
-    <t>2025-11-15T14:20:59Z</t>
-  </si>
-  <si>
-    <t>2025-11-14T19:56:55Z</t>
-  </si>
-  <si>
     <t>2026-06-17T18:46:10Z</t>
   </si>
   <si>
@@ -82,66 +82,66 @@
     <t>2026-06-17T22:43:35Z</t>
   </si>
   <si>
+    <t>2026-08-04T04:55:25Z</t>
+  </si>
+  <si>
+    <t>2026-09-01T02:17:13Z</t>
+  </si>
+  <si>
+    <t>2026-06-17T19:14:24Z</t>
+  </si>
+  <si>
+    <t>2026-07-16T15:26:02Z</t>
+  </si>
+  <si>
+    <t>2026-07-08T00:16:02Z</t>
+  </si>
+  <si>
+    <t>2026-06-13T11:04:18Z</t>
+  </si>
+  <si>
+    <t>2026-07-29T13:05:25Z</t>
+  </si>
+  <si>
+    <t>2025-11-05T10:38:10Z</t>
+  </si>
+  <si>
+    <t>2026-03-09T11:00:17Z</t>
+  </si>
+  <si>
     <t>2026-03-09T20:09:38Z</t>
   </si>
   <si>
-    <t>2026-03-09T11:00:17Z</t>
-  </si>
-  <si>
-    <t>2026-08-04T04:55:25Z</t>
-  </si>
-  <si>
-    <t>2026-06-17T19:14:24Z</t>
-  </si>
-  <si>
-    <t>2026-09-01T02:17:13Z</t>
-  </si>
-  <si>
-    <t>2026-07-08T00:16:02Z</t>
-  </si>
-  <si>
     <t>2025-11-05T10:38:09Z</t>
   </si>
   <si>
-    <t>2026-06-13T11:04:18Z</t>
-  </si>
-  <si>
-    <t>2025-11-05T10:38:10Z</t>
-  </si>
-  <si>
     <t>2026-03-10T14:29:11Z</t>
   </si>
   <si>
     <t>2026-03-10T08:42:36Z</t>
   </si>
   <si>
+    <t>2025-11-05T10:38:59Z</t>
+  </si>
+  <si>
+    <t>2026-06-18T11:33:52Z</t>
+  </si>
+  <si>
+    <t>2026-07-10T09:05:57Z</t>
+  </si>
+  <si>
+    <t>2026-03-10T08:15:12Z</t>
+  </si>
+  <si>
+    <t>2025-11-05T10:38:16Z</t>
+  </si>
+  <si>
+    <t>2026-06-17T19:09:58Z</t>
+  </si>
+  <si>
     <t>2026-06-07T10:33:42Z</t>
   </si>
   <si>
-    <t>2026-06-18T11:33:52Z</t>
-  </si>
-  <si>
-    <t>2025-11-05T10:38:59Z</t>
-  </si>
-  <si>
-    <t>2026-07-29T13:05:25Z</t>
-  </si>
-  <si>
-    <t>2026-07-10T09:05:57Z</t>
-  </si>
-  <si>
-    <t>2026-03-10T08:15:12Z</t>
-  </si>
-  <si>
-    <t>2025-11-05T10:38:16Z</t>
-  </si>
-  <si>
-    <t>2026-06-17T19:09:58Z</t>
-  </si>
-  <si>
-    <t>2026-07-16T15:26:02Z</t>
-  </si>
-  <si>
     <t>2025-11-15T12:04:28Z</t>
   </si>
   <si>
@@ -682,13 +682,16 @@
     <t>2025-11-15T19:24:30Z</t>
   </si>
   <si>
+    <t>['ftnctuniv:oai:ir.nctu.edu.tw:11536_63071']</t>
+  </si>
+  <si>
+    <t>['ftdoajarticles:oai:doaj.org_article:cbe415714bb341009a450266a64982b6']</t>
+  </si>
+  <si>
     <t>['ftdavidrumseyc:oai:N_A:RUMSEY~8~1~337492~90105339']</t>
   </si>
   <si>
-    <t>['ftnctuniv:oai:ir.nctu.edu.tw:11536_63071']</t>
-  </si>
-  <si>
-    <t>['ftdoajarticles:oai:doaj.org_article:cbe415714bb341009a450266a64982b6']</t>
+    <t>['ftunibolognairis:oai:cris.unibo.it:11585_743243', 'ftdoajarticles:oai:doaj.org_article:cbe415714bb341009a450266a64982b6']</t>
   </si>
   <si>
     <t>['ftumichgbhathi:oai:quod.lib.umich.edu:MIU01-102843695']</t>
@@ -700,69 +703,66 @@
     <t>['ftumichgbhathi:oai:quod.lib.umich.edu:MIU01-100235739']</t>
   </si>
   <si>
-    <t>['ftunibolognairis:oai:cris.unibo.it:11585_743243', 'ftdoajarticles:oai:doaj.org_article:cbe415714bb341009a450266a64982b6']</t>
-  </si>
-  <si>
     <t>['ftumichgbhathi:oai:quod.lib.umich.edu:MIU01-102316754']</t>
   </si>
   <si>
     <t>['ftunivromairis:oai:iris.uniroma1.it:11573_1509595']</t>
   </si>
   <si>
+    <t>['ftumichgbhathi:oai:quod.lib.umich.edu:MIU01-102829124']</t>
+  </si>
+  <si>
+    <t>['ftumichgbhathi:oai:quod.lib.umich.edu:MIU01-101686667']</t>
+  </si>
+  <si>
+    <t>['ftnorthwestusl:oai:scholarlycommons.law.northwestern.edu:njtip_symposium-1019']</t>
+  </si>
+  <si>
+    <t>['ftumichgbhathi:oai:quod.lib.umich.edu:MIU01-100851932']</t>
+  </si>
+  <si>
+    <t>['ftumichgbhathi:oai:quod.lib.umich.edu:MIU01-100239766']</t>
+  </si>
+  <si>
+    <t>['ftdergipark2ojs:oai:dergipark.org.tr:article_1502577']</t>
+  </si>
+  <si>
+    <t>['fttunivcrete:oai:dlib.tuc.gr:47531']</t>
+  </si>
+  <si>
+    <t>['fttunivcrete:oai:dlib.tuc.gr:58833']</t>
+  </si>
+  <si>
     <t>['fttunivcrete:oai:dlib.tuc.gr:54156']</t>
   </si>
   <si>
-    <t>['fttunivcrete:oai:dlib.tuc.gr:58833']</t>
-  </si>
-  <si>
-    <t>['ftumichgbhathi:oai:quod.lib.umich.edu:MIU01-102829124']</t>
-  </si>
-  <si>
-    <t>['ftumichgbhathi:oai:quod.lib.umich.edu:MIU01-101686667']</t>
-  </si>
-  <si>
-    <t>['ftumichgbhathi:oai:quod.lib.umich.edu:MIU01-100851932']</t>
-  </si>
-  <si>
-    <t>['fttunivcrete:oai:dlib.tuc.gr:47531']</t>
-  </si>
-  <si>
-    <t>['ftumichgbhathi:oai:quod.lib.umich.edu:MIU01-100239766']</t>
-  </si>
-  <si>
     <t>['fttunivcrete:oai:dlib.tuc.gr:96320']</t>
   </si>
   <si>
     <t>['ftumichgbhathi:oai:quod.lib.umich.edu:MIU01-007446622']</t>
   </si>
   <si>
+    <t>['fttunivcrete:oai:dlib.tuc.gr:85336']</t>
+  </si>
+  <si>
+    <t>['ftumichgbhathi:oai:quod.lib.umich.edu:MIU01-100236954']</t>
+  </si>
+  <si>
+    <t>['oai:library.oapen.org:20.500.12657_112677']</t>
+  </si>
+  <si>
+    <t>['fttunivcrete:oai:dlib.tuc.gr:74159']</t>
+  </si>
+  <si>
+    <t>['fttunivcrete:oai:dlib.tuc.gr:52197']</t>
+  </si>
+  <si>
+    <t>['ftumichgbhathi:oai:quod.lib.umich.edu:MIU01-101686667', 'ftumichgbhathi:oai:quod.lib.umich.edu:MIU01-101686667']</t>
+  </si>
+  <si>
     <t>['oai:library.oapen.org:20.500.12657_112633', 'ftoapen:oai:library.oapen.org:20.500.12657_112633']</t>
   </si>
   <si>
-    <t>['ftumichgbhathi:oai:quod.lib.umich.edu:MIU01-100236954']</t>
-  </si>
-  <si>
-    <t>['fttunivcrete:oai:dlib.tuc.gr:85336']</t>
-  </si>
-  <si>
-    <t>['ftdergipark2ojs:oai:dergipark.org.tr:article_1502577']</t>
-  </si>
-  <si>
-    <t>['oai:library.oapen.org:20.500.12657_112677']</t>
-  </si>
-  <si>
-    <t>['fttunivcrete:oai:dlib.tuc.gr:74159']</t>
-  </si>
-  <si>
-    <t>['fttunivcrete:oai:dlib.tuc.gr:52197']</t>
-  </si>
-  <si>
-    <t>['ftumichgbhathi:oai:quod.lib.umich.edu:MIU01-101686667', 'ftumichgbhathi:oai:quod.lib.umich.edu:MIU01-101686667']</t>
-  </si>
-  <si>
-    <t>['ftnorthwestusl:oai:scholarlycommons.law.northwestern.edu:njtip_symposium-1019']</t>
-  </si>
-  <si>
     <t>['ftunivtokyo:oai:repository.dl.itc.u-tokyo.ac.jp:00032435']</t>
   </si>
   <si>
@@ -1477,13 +1477,16 @@
     <t>['ftunivtokyo:oai:repository.dl.itc.u-tokyo.ac.jp:00029983']</t>
   </si>
   <si>
+    <t>['manag', 'eco']</t>
+  </si>
+  <si>
+    <t>['socio', 'demo']</t>
+  </si>
+  <si>
     <t>[]</t>
   </si>
   <si>
-    <t>['manag', 'eco']</t>
-  </si>
-  <si>
-    <t>['socio', 'demo']</t>
+    <t>['demo', 'envir', 'socio']</t>
   </si>
   <si>
     <t>['class', 'litt']</t>
@@ -1495,57 +1498,54 @@
     <t>['archi']</t>
   </si>
   <si>
-    <t>['demo', 'envir', 'socio']</t>
-  </si>
-  <si>
     <t>['info']</t>
   </si>
   <si>
     <t>['edu', 'psy']</t>
   </si>
   <si>
+    <t>['art', 'litt']</t>
+  </si>
+  <si>
+    <t>['art']</t>
+  </si>
+  <si>
+    <t>['droit', 'info']</t>
+  </si>
+  <si>
+    <t>['class']</t>
+  </si>
+  <si>
+    <t>['edu', 'info']</t>
+  </si>
+  <si>
+    <t>['info', 'demo', 'phil', 'edu']</t>
+  </si>
+  <si>
+    <t>['info', 'droit']</t>
+  </si>
+  <si>
     <t>['info', 'envir']</t>
   </si>
   <si>
-    <t>['info', 'droit']</t>
-  </si>
-  <si>
-    <t>['art', 'litt']</t>
-  </si>
-  <si>
-    <t>['art']</t>
-  </si>
-  <si>
-    <t>['info', 'demo', 'phil', 'edu']</t>
-  </si>
-  <si>
-    <t>['class']</t>
-  </si>
-  <si>
     <t>['eco', 'envir']</t>
   </si>
   <si>
     <t>['hist', 'hisphilso']</t>
   </si>
   <si>
+    <t>['lang', 'litt']</t>
+  </si>
+  <si>
+    <t>['info', 'geo']</t>
+  </si>
+  <si>
+    <t>['archeo', 'geo']</t>
+  </si>
+  <si>
     <t>['hist', 'scipo']</t>
   </si>
   <si>
-    <t>['edu', 'info']</t>
-  </si>
-  <si>
-    <t>['lang', 'litt']</t>
-  </si>
-  <si>
-    <t>['info', 'geo']</t>
-  </si>
-  <si>
-    <t>['archeo', 'geo']</t>
-  </si>
-  <si>
-    <t>['droit', 'info']</t>
-  </si>
-  <si>
     <t>['geo', 'demo']</t>
   </si>
   <si>
@@ -1900,16 +1900,19 @@
     <t>['hisphilso', 'psy']</t>
   </si>
   <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>11</t>
+  </si>
+  <si>
+    <t>4</t>
+  </si>
+  <si>
     <t>9</t>
   </si>
   <si>
-    <t>11</t>
-  </si>
-  <si>
-    <t>1</t>
-  </si>
-  <si>
-    <t>4</t>
+    <t>3</t>
   </si>
   <si>
     <t>Dante Alighieri, 1265-1321. De vulgari eloquentia. Italian. 1529. http://viaf.org/viaf/4668159477985727990005</t>
@@ -1921,9 +1924,6 @@
     <t>Vignola, 1507-1573. http://id.loc.gov/ities/names/n82222501 http://viaf.org/viaf/56637758</t>
   </si>
   <si>
-    <t>3</t>
-  </si>
-  <si>
     <t>Phillips, , auctioneer. http://id.loc.gov/ities/names/n83132163 http://viaf.org/viaf/75227852</t>
   </si>
   <si>
@@ -1933,72 +1933,72 @@
     <t>2019 at Uppsala Universitet BIBSAM http://jnnp. bmj. com/ J Neurol Neurosurg Psychiatry: first published as 10. 1136/jnnp-2019-321496 on 5 October 2019. Downloaded from 8 Verboon C</t>
   </si>
   <si>
+    <t>Hunter, Aaron Burtis, 1854-1933, http://id.loc.gov/ities/names/no2010024138 former owner.</t>
+  </si>
+  <si>
+    <t>Bloemaert, Abraham, 1564-1651 http://id.loc.gov/ities/names/nr93052276 http://viaf.org/viaf/77114225</t>
+  </si>
+  <si>
+    <t>Sponsored by Northwestern Law School’s Master of Science in Law, a one-year Master’s degree in law for scientists and engineers. For more information, please visit: http://www.law.northwestern.edu/academics/degree-programs/msl</t>
+  </si>
+  <si>
+    <t>Bosse, Abraham, 1602-1676 http://id.loc.gov/ities/names/n82272447 http://viaf.org/viaf/61542289</t>
+  </si>
+  <si>
+    <t>Bocchi, Achille, 1488-1562 http://id.loc.gov/ities/names/n92057019 http://viaf.org/viaf/149878</t>
+  </si>
+  <si>
+    <t>Http://2024.brs.org.tr, Abstract Book Of 8th International Brain Research School 20 - 26 May 2024, Isparta /türkiye.</t>
+  </si>
+  <si>
+    <t>Aggelakis Dimitrios(http://users.isc.tuc.gr/~daggelakis)</t>
+  </si>
+  <si>
+    <t>Qiao Li, 1934-(http://viaf.org/viaf/112423839)</t>
+  </si>
+  <si>
+    <t>Moropoulou, A(http://viaf.org/viaf/305714749)</t>
+  </si>
+  <si>
     <t>Bakolas, A(http://viaf.org/viaf/305714756)</t>
   </si>
   <si>
-    <t>Qiao Li, 1934-(http://viaf.org/viaf/112423839)</t>
-  </si>
-  <si>
-    <t>Moropoulou, A(http://viaf.org/viaf/305714749)</t>
-  </si>
-  <si>
-    <t>Hunter, Aaron Burtis, 1854-1933, http://id.loc.gov/ities/names/no2010024138 former owner.</t>
-  </si>
-  <si>
-    <t>Bloemaert, Abraham, 1564-1651 http://id.loc.gov/ities/names/nr93052276 http://viaf.org/viaf/77114225</t>
-  </si>
-  <si>
-    <t>Bosse, Abraham, 1602-1676 http://id.loc.gov/ities/names/n82272447 http://viaf.org/viaf/61542289</t>
-  </si>
-  <si>
     <t>Αγγελακης Δημητριος(http://users.isc.tuc.gr/~daggelakis)</t>
   </si>
   <si>
-    <t>Bocchi, Achille, 1488-1562 http://id.loc.gov/ities/names/n92057019 http://viaf.org/viaf/149878</t>
-  </si>
-  <si>
-    <t>Aggelakis Dimitrios(http://users.isc.tuc.gr/~daggelakis)</t>
+    <t>Ακασιαδης Χαριλαος(http://users.isc.tuc.gr/~cakasiadis)</t>
   </si>
   <si>
     <t>Akasiadis Charilaos(http://users.isc.tuc.gr/~cakasiadis)</t>
   </si>
   <si>
-    <t>Ακασιαδης Χαριλαος(http://users.isc.tuc.gr/~cakasiadis)</t>
-  </si>
-  <si>
     <t>Macquarrie, Alan (Alan Denis), . http://id.loc.gov/ities/names/n85098805</t>
   </si>
   <si>
+    <t>Αλεβιζος Παναγιωτης(http://users.isc.tuc.gr/~palevizos)</t>
+  </si>
+  <si>
+    <t>Alevizos Panagiotis(http://users.isc.tuc.gr/~palevizos)</t>
+  </si>
+  <si>
+    <t>Dürer, Albrecht, 1471-1528 http://id.loc.gov/ities/names/n79118011 http://viaf.org/viaf/54146999</t>
+  </si>
+  <si>
+    <t>Troy L. Cox - http://.org/0000-0001-9379-5102, Alan V. Brown - http://.org/0000-0003-0144-4722,Margaret E. Malone - http://.org/0000-0001-9640-412X</t>
+  </si>
+  <si>
+    <t>Artikis, Alexander(http://viaf.org/viaf/43834206)</t>
+  </si>
+  <si>
+    <t>Sarris, Alexander(http://viaf.org/viaf/19743442)</t>
+  </si>
+  <si>
+    <t>Browne, Alexander, active 1660-1677 http://id.loc.gov/ities/names/n85035349 http://viaf.org/viaf/22988134</t>
+  </si>
+  <si>
     <t>Ayyad , Ahmad | http://.org/0009-0007-2829-2382</t>
   </si>
   <si>
-    <t>Dürer, Albrecht, 1471-1528 http://id.loc.gov/ities/names/n79118011 http://viaf.org/viaf/54146999</t>
-  </si>
-  <si>
-    <t>Αλεβιζος Παναγιωτης(http://users.isc.tuc.gr/~palevizos)</t>
-  </si>
-  <si>
-    <t>Http://2024.brs.org.tr, Abstract Book Of 8th International Brain Research School 20 - 26 May 2024, Isparta /türkiye.</t>
-  </si>
-  <si>
-    <t>Alevizos Panagiotis(http://users.isc.tuc.gr/~palevizos)</t>
-  </si>
-  <si>
-    <t>Troy L. Cox - http://.org/0000-0001-9379-5102, Alan V. Brown - http://.org/0000-0003-0144-4722,Margaret E. Malone - http://.org/0000-0001-9640-412X</t>
-  </si>
-  <si>
-    <t>Artikis, Alexander(http://viaf.org/viaf/43834206)</t>
-  </si>
-  <si>
-    <t>Sarris, Alexander(http://viaf.org/viaf/19743442)</t>
-  </si>
-  <si>
-    <t>Browne, Alexander, active 1660-1677 http://id.loc.gov/ities/names/n85035349 http://viaf.org/viaf/22988134</t>
-  </si>
-  <si>
-    <t>Sponsored by Northwestern Law School’s Master of Science in Law, a one-year Master’s degree in law for scientists and engineers. For more information, please visit: http://www.law.northwestern.edu/academics/degree-programs/msl</t>
-  </si>
-  <si>
     <t>123598</t>
   </si>
   <si>
@@ -3415,82 +3415,85 @@
     <t>2019 At Uppsala Universitet Bibsam  Bmj. Com  J Neurol Neurosurg Psychiatry  First Published As 10. 1136 Jnnp-2019-321496 On 5 October 2019. Downloaded From 8 Verboon C</t>
   </si>
   <si>
+    <t>Hunter, Aaron Burtis, 1854-1933,  Former Owner.</t>
+  </si>
+  <si>
+    <t>Bloemaert, Abraham, 1564-1651</t>
+  </si>
+  <si>
+    <t>Sponsored By Northwestern Law School’S Master Of Science In Law, A One-Year Master’S Degree In Law For Scientists And Engineers. For More Information, Please Visit</t>
+  </si>
+  <si>
+    <t>Bosse, Abraham, 1602-1676</t>
+  </si>
+  <si>
+    <t>Bocchi, Achille, 1488-1562</t>
+  </si>
+  <si>
+    <t>Http 2024.Brs.Org.Tr, Abstract Book Of 8Th International Brain Research School 20 - 26 May 2024, Isparta  Türkiye.</t>
+  </si>
+  <si>
+    <t>Aggelakis Dimitrios(</t>
+  </si>
+  <si>
+    <t>Qiao Li, 1934-(</t>
+  </si>
+  <si>
+    <t>Moropoulou, A(</t>
+  </si>
+  <si>
     <t>Bakolas, A(</t>
   </si>
   <si>
-    <t>Qiao Li, 1934-(</t>
-  </si>
-  <si>
-    <t>Moropoulou, A(</t>
-  </si>
-  <si>
-    <t>Hunter, Aaron Burtis, 1854-1933,  Former Owner.</t>
-  </si>
-  <si>
-    <t>Bloemaert, Abraham, 1564-1651</t>
-  </si>
-  <si>
-    <t>Bosse, Abraham, 1602-1676</t>
-  </si>
-  <si>
     <t>Αγγελακης Δημητριος(</t>
   </si>
   <si>
-    <t>Bocchi, Achille, 1488-1562</t>
-  </si>
-  <si>
-    <t>Aggelakis Dimitrios(</t>
+    <t>Ακασιαδης Χαριλαος(</t>
   </si>
   <si>
     <t>Akasiadis Charilaos(</t>
   </si>
   <si>
-    <t>Ακασιαδης Χαριλαος(</t>
-  </si>
-  <si>
     <t>Macquarrie, Alan (Alan Denis), .</t>
   </si>
   <si>
+    <t>Αλεβιζος Παναγιωτης(</t>
+  </si>
+  <si>
+    <t>Alevizos Panagiotis(</t>
+  </si>
+  <si>
+    <t>DüRer, Albrecht, 1471-1528</t>
+  </si>
+  <si>
+    <t>Troy L. Cox</t>
+  </si>
+  <si>
+    <t>Artikis, Alexander(</t>
+  </si>
+  <si>
+    <t>Sarris, Alexander(</t>
+  </si>
+  <si>
+    <t>Browne, Alexander, Active 1660-1677</t>
+  </si>
+  <si>
     <t>Ahmad Ayyad</t>
   </si>
   <si>
-    <t>DüRer, Albrecht, 1471-1528</t>
-  </si>
-  <si>
-    <t>Αλεβιζος Παναγιωτης(</t>
-  </si>
-  <si>
-    <t>Http 2024.Brs.Org.Tr, Abstract Book Of 8Th International Brain Research School 20 - 26 May 2024, Isparta  Türkiye.</t>
-  </si>
-  <si>
-    <t>Alevizos Panagiotis(</t>
-  </si>
-  <si>
-    <t>Troy L. Cox</t>
-  </si>
-  <si>
-    <t>Artikis, Alexander(</t>
-  </si>
-  <si>
-    <t>Sarris, Alexander(</t>
-  </si>
-  <si>
-    <t>Browne, Alexander, Active 1660-1677</t>
-  </si>
-  <si>
-    <t>Sponsored By Northwestern Law School’S Master Of Science In Law, A One-Year Master’S Degree In Law For Scientists And Engineers. For More Information, Please Visit</t>
+    <t>__Qb6dhGCuSF8a_Zyxy01hJ</t>
+  </si>
+  <si>
+    <t>__Lf3PykJx4L9-dTyQMzBbm</t>
+  </si>
+  <si>
+    <t>__oC9E7cVS7fOxYjgW1atqq</t>
   </si>
   <si>
     <t>__rYNuWw1igYZC1D8Zc0ebE</t>
   </si>
   <si>
-    <t>__Lf3PykJx4L9-dTyQMzBbm</t>
-  </si>
-  <si>
-    <t>__Qb6dhGCuSF8a_Zyxy01hJ</t>
-  </si>
-  <si>
-    <t>__oC9E7cVS7fOxYjgW1atqq</t>
+    <t>__e6hWqSg7_qiy0-u-Y4F8J</t>
   </si>
   <si>
     <t>_de_vulgari_eloquentia_italian_http_viaf_org_viaf_dante_alighieri_1qjOi8VRcChBfdjgLHEvW</t>
@@ -3502,9 +3505,6 @@
     <t>_http_id_loc_gov_ities_names_n_http_viaf_org_viaf_vignola_4a9lrp9xVMnfJnEld9bIm</t>
   </si>
   <si>
-    <t>__e6hWqSg7_qiy0-u-Y4F8J</t>
-  </si>
-  <si>
     <t>_phillips_xL_mm5joH8RR8NN9FwRss</t>
   </si>
   <si>
@@ -3514,75 +3514,75 @@
     <t>_at_uppsala_universitet_bibsam_http_jnnp_bmj_com_j_neurol_neurosurg_psychiatry_first_published_as_jnnp_on_october_downloaded_from_verboon_c_RuaF0aB-PREMU0qSv6bqi</t>
   </si>
   <si>
+    <t>aaron_burtis_hunter_5-uNyPpE5Chfzp3N6hX2K</t>
+  </si>
+  <si>
+    <t>aaron_burtis_hunter__F094Vs8Kn3yYvsbsz5Rb</t>
+  </si>
+  <si>
+    <t>abraham_bloemaert_oZ6C8dT3gphESC3accfhB</t>
+  </si>
+  <si>
+    <t>a_one_year_master_s_degree_in_law_for_scientists_and_engineers_for_more_information_sponsored_by_northwestern_law_school_s_master_of_science_in_law_8efEG1i5djhXfS0SKuS-l</t>
+  </si>
+  <si>
+    <t>abraham_bosse_zUWLzd5Tzlo6G31QJWjpS</t>
+  </si>
+  <si>
+    <t>achille_bocchi_UqHriJVSjpVKFq_wiX5Ft</t>
+  </si>
+  <si>
+    <t>abstract_book_of_th_international_brain_research_school_may_http_brs_org_tr_0rM1E8eCsvR_nWDwnb6vS</t>
+  </si>
+  <si>
+    <t>aggelakis_dimitrios_http_usersisctucgr_daggelakis__jIc5BseH9b-LU4DEaS0ba</t>
+  </si>
+  <si>
+    <t>_http_viaf_org_viaf_qiao_li_bk7_1hQX8nv0OwhQOMk3Q</t>
+  </si>
+  <si>
+    <t>a_http_viaf_org_viaf_moropoulou_8vc8YnjwfWJSOjaMqXu6D</t>
+  </si>
+  <si>
     <t>a_http_viaf_org_viaf_bakolas_0GqmLcGsS7C7WLSL3Uqb-</t>
   </si>
   <si>
-    <t>_http_viaf_org_viaf_qiao_li_bk7_1hQX8nv0OwhQOMk3Q</t>
-  </si>
-  <si>
-    <t>a_http_viaf_org_viaf_moropoulou_8vc8YnjwfWJSOjaMqXu6D</t>
-  </si>
-  <si>
-    <t>aaron_burtis_hunter_5-uNyPpE5Chfzp3N6hX2K</t>
-  </si>
-  <si>
-    <t>abraham_bloemaert_oZ6C8dT3gphESC3accfhB</t>
-  </si>
-  <si>
-    <t>aaron_burtis_hunter__F094Vs8Kn3yYvsbsz5Rb</t>
-  </si>
-  <si>
-    <t>abraham_bosse_zUWLzd5Tzlo6G31QJWjpS</t>
-  </si>
-  <si>
     <t>aggelakes_demetrios_http_usersisctucgr_daggelakis__XaAsKWahng05KEm2pWq5M</t>
   </si>
   <si>
-    <t>achille_bocchi_UqHriJVSjpVKFq_wiX5Ft</t>
-  </si>
-  <si>
-    <t>aggelakis_dimitrios_http_usersisctucgr_daggelakis__jIc5BseH9b-LU4DEaS0ba</t>
+    <t>akasiades_kharilaos_http_usersisctucgr_cakasiadis__IgSIifR7F6n5pt5ZrNEmB</t>
   </si>
   <si>
     <t>akasiadis_charilaos_http_usersisctucgr_cakasiadis__riy2zSfSLEPuWrGxmW39K</t>
   </si>
   <si>
-    <t>akasiades_kharilaos_http_usersisctucgr_cakasiadis__IgSIifR7F6n5pt5ZrNEmB</t>
-  </si>
-  <si>
     <t>alan_alan_denis_macquarrie_LKNnU5RopnZ7OEIuOX_oO</t>
   </si>
   <si>
+    <t>alebizos_panagiotes_http_usersisctucgr_palevizos__dRBO8_6ZVWVnUYetze1Sk</t>
+  </si>
+  <si>
+    <t>alevizos_panagiotis_http_usersisctucgr_palevizos__iyh5iJoRgapvpC1Xi_No8</t>
+  </si>
+  <si>
+    <t>albrecht_durer_beP_z8DGp_ecqp2zvWIOL</t>
+  </si>
+  <si>
+    <t>alan_v_brown_http_org_troy_l_cox_http_org__C8vYqCZfeLBuEzh2HIDl0</t>
+  </si>
+  <si>
+    <t>alexander_http_viaf_org_viaf_artikis_GBrdqjHsf5aeL3_JWbdZX</t>
+  </si>
+  <si>
+    <t>alexander_http_viaf_org_viaf_sarris_T8gPE2F4bSlOQWScIWObS</t>
+  </si>
+  <si>
+    <t>alexander_browne_kCJZhQLRS66FZrQCsYyvq</t>
+  </si>
+  <si>
     <t>ahmad_http_org_ayyad_tXusKa1yR1zW6CupaZJMG</t>
   </si>
   <si>
-    <t>albrecht_durer_beP_z8DGp_ecqp2zvWIOL</t>
-  </si>
-  <si>
-    <t>alebizos_panagiotes_http_usersisctucgr_palevizos__dRBO8_6ZVWVnUYetze1Sk</t>
-  </si>
-  <si>
-    <t>abstract_book_of_th_international_brain_research_school_may_http_brs_org_tr_0rM1E8eCsvR_nWDwnb6vS</t>
-  </si>
-  <si>
-    <t>alevizos_panagiotis_http_usersisctucgr_palevizos__iyh5iJoRgapvpC1Xi_No8</t>
-  </si>
-  <si>
-    <t>alan_v_brown_http_org_troy_l_cox_http_org__C8vYqCZfeLBuEzh2HIDl0</t>
-  </si>
-  <si>
-    <t>alexander_http_viaf_org_viaf_artikis_GBrdqjHsf5aeL3_JWbdZX</t>
-  </si>
-  <si>
-    <t>alexander_http_viaf_org_viaf_sarris_T8gPE2F4bSlOQWScIWObS</t>
-  </si>
-  <si>
-    <t>alexander_browne_kCJZhQLRS66FZrQCsYyvq</t>
-  </si>
-  <si>
-    <t>a_one_year_master_s_degree_in_law_for_scientists_and_engineers_for_more_information_sponsored_by_northwestern_law_school_s_master_of_science_in_law_8efEG1i5djhXfS0SKuS-l</t>
-  </si>
-  <si>
     <t>__-76q-D_tyR-oRhWq8F96z</t>
   </si>
   <si>
@@ -4981,10 +4981,10 @@
     <t>__zp9Yp5_EPKG_1b2bcs4gK</t>
   </si>
   <si>
+    <t>0000-0001-9379-5102</t>
+  </si>
+  <si>
     <t>0009-0007-2829-2382</t>
-  </si>
-  <si>
-    <t>0000-0001-9379-5102</t>
   </si>
   <si>
     <t>numeric</t>
@@ -6570,13 +6570,13 @@
     </row>
     <row r="3" spans="1:13">
       <c r="A3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B3" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="C3" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="D3">
         <v>2</v>
@@ -6675,7 +6675,7 @@
     </row>
     <row r="6" spans="1:13">
       <c r="A6" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B6" t="s">
         <v>225</v>
@@ -6684,33 +6684,33 @@
         <v>490</v>
       </c>
       <c r="D6">
-        <v>109</v>
+        <v>1</v>
       </c>
       <c r="E6" t="s">
         <v>632</v>
       </c>
       <c r="F6" t="s">
-        <v>1127</v>
+        <v>632</v>
       </c>
       <c r="G6" t="s">
         <v>1159</v>
       </c>
       <c r="I6">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J6" t="b">
         <v>0</v>
       </c>
       <c r="K6" t="s">
-        <v>1658</v>
+        <v>1657</v>
       </c>
       <c r="L6" t="s">
-        <v>1661</v>
+        <v>1660</v>
       </c>
     </row>
     <row r="7" spans="1:13">
       <c r="A7" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B7" t="s">
         <v>226</v>
@@ -6719,13 +6719,13 @@
         <v>491</v>
       </c>
       <c r="D7">
-        <v>119</v>
+        <v>109</v>
       </c>
       <c r="E7" t="s">
         <v>633</v>
       </c>
       <c r="F7" t="s">
-        <v>1128</v>
+        <v>1127</v>
       </c>
       <c r="G7" t="s">
         <v>1160</v>
@@ -6745,7 +6745,7 @@
     </row>
     <row r="8" spans="1:13">
       <c r="A8" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B8" t="s">
         <v>227</v>
@@ -6754,13 +6754,13 @@
         <v>492</v>
       </c>
       <c r="D8">
-        <v>89</v>
+        <v>119</v>
       </c>
       <c r="E8" t="s">
         <v>634</v>
       </c>
       <c r="F8" t="s">
-        <v>1129</v>
+        <v>1128</v>
       </c>
       <c r="G8" t="s">
         <v>1161</v>
@@ -6780,7 +6780,7 @@
     </row>
     <row r="9" spans="1:13">
       <c r="A9" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="B9" t="s">
         <v>228</v>
@@ -6789,28 +6789,28 @@
         <v>493</v>
       </c>
       <c r="D9">
-        <v>1</v>
+        <v>89</v>
       </c>
       <c r="E9" t="s">
         <v>635</v>
       </c>
       <c r="F9" t="s">
-        <v>635</v>
+        <v>1129</v>
       </c>
       <c r="G9" t="s">
         <v>1162</v>
       </c>
       <c r="I9">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J9" t="b">
         <v>0</v>
       </c>
       <c r="K9" t="s">
-        <v>1657</v>
+        <v>1658</v>
       </c>
       <c r="L9" t="s">
-        <v>1660</v>
+        <v>1661</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -6853,10 +6853,10 @@
         <v>20</v>
       </c>
       <c r="B11" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="C11" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
       <c r="D11">
         <v>87</v>
@@ -6929,7 +6929,7 @@
         <v>496</v>
       </c>
       <c r="D13">
-        <v>42</v>
+        <v>89</v>
       </c>
       <c r="E13" t="s">
         <v>639</v>
@@ -6958,19 +6958,19 @@
         <v>23</v>
       </c>
       <c r="B14" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="C14" t="s">
-        <v>497</v>
+        <v>496</v>
       </c>
       <c r="D14">
-        <v>46</v>
+        <v>89</v>
       </c>
       <c r="E14" t="s">
-        <v>640</v>
+        <v>639</v>
       </c>
       <c r="F14" t="s">
-        <v>1134</v>
+        <v>1133</v>
       </c>
       <c r="G14" t="s">
         <v>1167</v>
@@ -6990,22 +6990,22 @@
     </row>
     <row r="15" spans="1:13">
       <c r="A15" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B15" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="C15" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="D15">
-        <v>45</v>
+        <v>100</v>
       </c>
       <c r="E15" t="s">
-        <v>641</v>
+        <v>640</v>
       </c>
       <c r="F15" t="s">
-        <v>1135</v>
+        <v>1134</v>
       </c>
       <c r="G15" t="s">
         <v>1168</v>
@@ -7025,7 +7025,7 @@
     </row>
     <row r="16" spans="1:13">
       <c r="A16" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B16" t="s">
         <v>233</v>
@@ -7034,13 +7034,13 @@
         <v>498</v>
       </c>
       <c r="D16">
-        <v>89</v>
+        <v>226</v>
       </c>
       <c r="E16" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="F16" t="s">
-        <v>1136</v>
+        <v>1135</v>
       </c>
       <c r="G16" t="s">
         <v>1169</v>
@@ -7060,22 +7060,22 @@
     </row>
     <row r="17" spans="1:12">
       <c r="A17" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B17" t="s">
         <v>234</v>
       </c>
       <c r="C17" t="s">
-        <v>499</v>
+        <v>492</v>
       </c>
       <c r="D17">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="E17" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="F17" t="s">
-        <v>1137</v>
+        <v>1136</v>
       </c>
       <c r="G17" t="s">
         <v>1170</v>
@@ -7095,22 +7095,22 @@
     </row>
     <row r="18" spans="1:12">
       <c r="A18" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B18" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="C18" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="D18">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="E18" t="s">
-        <v>642</v>
+        <v>643</v>
       </c>
       <c r="F18" t="s">
-        <v>1136</v>
+        <v>1137</v>
       </c>
       <c r="G18" t="s">
         <v>1171</v>
@@ -7130,16 +7130,16 @@
     </row>
     <row r="19" spans="1:12">
       <c r="A19" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B19" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="C19" t="s">
-        <v>491</v>
+        <v>500</v>
       </c>
       <c r="D19">
-        <v>95</v>
+        <v>116</v>
       </c>
       <c r="E19" t="s">
         <v>644</v>
@@ -7165,13 +7165,13 @@
     </row>
     <row r="20" spans="1:12">
       <c r="A20" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B20" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="C20" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="D20">
         <v>56</v>
@@ -7200,16 +7200,16 @@
     </row>
     <row r="21" spans="1:12">
       <c r="A21" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B21" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="C21" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="D21">
-        <v>94</v>
+        <v>46</v>
       </c>
       <c r="E21" t="s">
         <v>646</v>
@@ -7235,16 +7235,16 @@
     </row>
     <row r="22" spans="1:12">
       <c r="A22" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B22" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="C22" t="s">
-        <v>500</v>
+        <v>503</v>
       </c>
       <c r="D22">
-        <v>56</v>
+        <v>45</v>
       </c>
       <c r="E22" t="s">
         <v>647</v>
@@ -7273,13 +7273,13 @@
         <v>31</v>
       </c>
       <c r="B23" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="C23" t="s">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="D23">
-        <v>56</v>
+        <v>42</v>
       </c>
       <c r="E23" t="s">
         <v>648</v>
@@ -7305,16 +7305,16 @@
     </row>
     <row r="24" spans="1:12">
       <c r="A24" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B24" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="C24" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="D24">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E24" t="s">
         <v>649</v>
@@ -7340,16 +7340,16 @@
     </row>
     <row r="25" spans="1:12">
       <c r="A25" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B25" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="C25" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="D25">
-        <v>72</v>
+        <v>55</v>
       </c>
       <c r="E25" t="s">
         <v>650</v>
@@ -7384,7 +7384,7 @@
         <v>504</v>
       </c>
       <c r="D26">
-        <v>47</v>
+        <v>56</v>
       </c>
       <c r="E26" t="s">
         <v>651</v>
@@ -7395,20 +7395,17 @@
       <c r="G26" t="s">
         <v>1179</v>
       </c>
-      <c r="H26" t="s">
-        <v>1655</v>
-      </c>
       <c r="I26">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J26" t="b">
         <v>0</v>
       </c>
       <c r="K26" t="s">
-        <v>1659</v>
+        <v>1658</v>
       </c>
       <c r="L26" t="s">
-        <v>1662</v>
+        <v>1661</v>
       </c>
     </row>
     <row r="27" spans="1:12">
@@ -7419,10 +7416,10 @@
         <v>241</v>
       </c>
       <c r="C27" t="s">
-        <v>487</v>
+        <v>505</v>
       </c>
       <c r="D27">
-        <v>97</v>
+        <v>72</v>
       </c>
       <c r="E27" t="s">
         <v>652</v>
@@ -7483,16 +7480,16 @@
     </row>
     <row r="29" spans="1:12">
       <c r="A29" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B29" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="C29" t="s">
-        <v>505</v>
+        <v>494</v>
       </c>
       <c r="D29">
-        <v>116</v>
+        <v>55</v>
       </c>
       <c r="E29" t="s">
         <v>654</v>
@@ -7518,16 +7515,16 @@
     </row>
     <row r="30" spans="1:12">
       <c r="A30" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B30" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="C30" t="s">
-        <v>494</v>
+        <v>489</v>
       </c>
       <c r="D30">
-        <v>55</v>
+        <v>97</v>
       </c>
       <c r="E30" t="s">
         <v>655</v>
@@ -7574,7 +7571,7 @@
         <v>1184</v>
       </c>
       <c r="H31" t="s">
-        <v>1656</v>
+        <v>1655</v>
       </c>
       <c r="I31">
         <v>1</v>
@@ -7667,7 +7664,7 @@
         <v>247</v>
       </c>
       <c r="C34" t="s">
-        <v>499</v>
+        <v>497</v>
       </c>
       <c r="D34">
         <v>105</v>
@@ -7705,7 +7702,7 @@
         <v>509</v>
       </c>
       <c r="D35">
-        <v>226</v>
+        <v>47</v>
       </c>
       <c r="E35" t="s">
         <v>660</v>
@@ -7716,17 +7713,20 @@
       <c r="G35" t="s">
         <v>1188</v>
       </c>
+      <c r="H35" t="s">
+        <v>1656</v>
+      </c>
       <c r="I35">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J35" t="b">
         <v>0</v>
       </c>
       <c r="K35" t="s">
-        <v>1658</v>
+        <v>1659</v>
       </c>
       <c r="L35" t="s">
-        <v>1661</v>
+        <v>1662</v>
       </c>
     </row>
     <row r="36" spans="1:13">
@@ -7927,7 +7927,7 @@
         <v>254</v>
       </c>
       <c r="C41" t="s">
-        <v>505</v>
+        <v>500</v>
       </c>
       <c r="D41">
         <v>6</v>
@@ -8079,7 +8079,7 @@
         <v>254</v>
       </c>
       <c r="C45" t="s">
-        <v>505</v>
+        <v>500</v>
       </c>
       <c r="D45">
         <v>6</v>
@@ -8497,7 +8497,7 @@
         <v>267</v>
       </c>
       <c r="C56" t="s">
-        <v>498</v>
+        <v>496</v>
       </c>
       <c r="D56">
         <v>6</v>
@@ -8573,7 +8573,7 @@
         <v>269</v>
       </c>
       <c r="C58" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="D58">
         <v>5</v>
@@ -9105,7 +9105,7 @@
         <v>281</v>
       </c>
       <c r="C72" t="s">
-        <v>504</v>
+        <v>509</v>
       </c>
       <c r="D72">
         <v>5</v>
@@ -10017,7 +10017,7 @@
         <v>302</v>
       </c>
       <c r="C96" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="D96">
         <v>6</v>
@@ -10055,7 +10055,7 @@
         <v>281</v>
       </c>
       <c r="C97" t="s">
-        <v>504</v>
+        <v>509</v>
       </c>
       <c r="D97">
         <v>5</v>
@@ -11005,7 +11005,7 @@
         <v>281</v>
       </c>
       <c r="C122" t="s">
-        <v>504</v>
+        <v>509</v>
       </c>
       <c r="D122">
         <v>5</v>
@@ -11613,7 +11613,7 @@
         <v>329</v>
       </c>
       <c r="C138" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="D138">
         <v>6</v>
@@ -11841,7 +11841,7 @@
         <v>334</v>
       </c>
       <c r="C144" t="s">
-        <v>509</v>
+        <v>498</v>
       </c>
       <c r="D144">
         <v>5</v>
@@ -11993,7 +11993,7 @@
         <v>337</v>
       </c>
       <c r="C148" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="D148">
         <v>5</v>
@@ -12107,7 +12107,7 @@
         <v>339</v>
       </c>
       <c r="C151" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="D151">
         <v>5</v>
@@ -12981,7 +12981,7 @@
         <v>355</v>
       </c>
       <c r="C174" t="s">
-        <v>502</v>
+        <v>504</v>
       </c>
       <c r="D174">
         <v>5</v>
@@ -13475,7 +13475,7 @@
         <v>254</v>
       </c>
       <c r="C187" t="s">
-        <v>505</v>
+        <v>500</v>
       </c>
       <c r="D187">
         <v>6</v>
@@ -13665,7 +13665,7 @@
         <v>364</v>
       </c>
       <c r="C192" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="D192">
         <v>5</v>
@@ -14273,7 +14273,7 @@
         <v>281</v>
       </c>
       <c r="C208" t="s">
-        <v>504</v>
+        <v>509</v>
       </c>
       <c r="D208">
         <v>5</v>
@@ -14653,7 +14653,7 @@
         <v>254</v>
       </c>
       <c r="C218" t="s">
-        <v>505</v>
+        <v>500</v>
       </c>
       <c r="D218">
         <v>6</v>
@@ -14805,7 +14805,7 @@
         <v>269</v>
       </c>
       <c r="C222" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="D222">
         <v>5</v>
@@ -15679,7 +15679,7 @@
         <v>254</v>
       </c>
       <c r="C245" t="s">
-        <v>505</v>
+        <v>500</v>
       </c>
       <c r="D245">
         <v>6</v>
@@ -16591,7 +16591,7 @@
         <v>302</v>
       </c>
       <c r="C269" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="D269">
         <v>6</v>
@@ -17389,7 +17389,7 @@
         <v>254</v>
       </c>
       <c r="C290" t="s">
-        <v>505</v>
+        <v>500</v>
       </c>
       <c r="D290">
         <v>6</v>
@@ -17655,7 +17655,7 @@
         <v>411</v>
       </c>
       <c r="C297" t="s">
-        <v>504</v>
+        <v>509</v>
       </c>
       <c r="D297">
         <v>5</v>
@@ -20163,7 +20163,7 @@
         <v>434</v>
       </c>
       <c r="C363" t="s">
-        <v>505</v>
+        <v>500</v>
       </c>
       <c r="D363">
         <v>6</v>
@@ -20467,7 +20467,7 @@
         <v>364</v>
       </c>
       <c r="C371" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="D371">
         <v>5</v>
@@ -20657,7 +20657,7 @@
         <v>254</v>
       </c>
       <c r="C376" t="s">
-        <v>505</v>
+        <v>500</v>
       </c>
       <c r="D376">
         <v>6</v>
@@ -21037,7 +21037,7 @@
         <v>254</v>
       </c>
       <c r="C386" t="s">
-        <v>505</v>
+        <v>500</v>
       </c>
       <c r="D386">
         <v>6</v>
@@ -21189,7 +21189,7 @@
         <v>440</v>
       </c>
       <c r="C390" t="s">
-        <v>504</v>
+        <v>509</v>
       </c>
       <c r="D390">
         <v>5</v>
@@ -21531,7 +21531,7 @@
         <v>254</v>
       </c>
       <c r="C399" t="s">
-        <v>505</v>
+        <v>500</v>
       </c>
       <c r="D399">
         <v>6</v>
@@ -21721,7 +21721,7 @@
         <v>446</v>
       </c>
       <c r="C404" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="D404">
         <v>5</v>
@@ -22139,7 +22139,7 @@
         <v>453</v>
       </c>
       <c r="C415" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="D415">
         <v>6</v>
@@ -22405,7 +22405,7 @@
         <v>455</v>
       </c>
       <c r="C422" t="s">
-        <v>504</v>
+        <v>509</v>
       </c>
       <c r="D422">
         <v>5</v>

</xml_diff>